<commit_message>
corrected behavior in handling changes to input xlsx, was creating duplicates before, is not now. Additionally, added function using input from terminal to de-duplicate any places where the name was changed (intentionally or not). This is the only place where it cannot be handled dynamically in the program because the pipeline assumes the name of the place is the source of truth and not a typo.
</commit_message>
<xml_diff>
--- a/ATL-Food-and-Drink-Review-List.xlsx
+++ b/ATL-Food-and-Drink-Review-List.xlsx
@@ -738,7 +738,7 @@
     <t>5090 Buford Hwy, Doraville, GA 30340</t>
   </si>
   <si>
-    <t>J’s Mini Hot Pot</t>
+    <t>J's Mini Hot Pot</t>
   </si>
   <si>
     <t>farthest, chamblee location just closed :( each person gets their own mini hot pot</t>
@@ -1413,7 +1413,7 @@
     <t>4897 Buford Hwy #109, Chamblee, GA 30341</t>
   </si>
   <si>
-    <t>Gu’s Kitchen</t>
+    <t>Gu's Kitchen</t>
   </si>
   <si>
     <t>Brick and mortar location (dumpling stall in Krog). String beans were fantastic. Prices were a bit high but food was delicious</t>

</xml_diff>